<commit_message>
Rebalance evidence: trim redundant Ethan items, add noise, soften naming
- Dropped 4 redundant Ethan items (E03, E05, E26, E27) that repeated the
  same "record proves the credential/account, not the person" point;
  Ethan's count goes from 13 to 9, closer to everyone else's ~6.
- Added 5 new low-relevance/red-herring items (delivery, rumor, HVAC
  quirk, unrelated visitor badge, unrelated old incident) that don't
  point anywhere, to dilute the signal-to-noise ratio. Total evidence
  is now 33.
- Reworded the top-level (pre-Dig-In) line for the motive/character
  items (E01, E22, E23, E24, E29, E30, E31) to describe a role instead
  of naming the suspect outright, e.g. "The lead researcher opposed..."
  instead of "Ethan opposed...". Digging in is what actually surfaces
  the name — system-log lines (badge/account/device entries) are left
  named since a real access log inherently shows whose credential it is.
- Re-ran the board-spread scheduler over the new 33-item set.
</commit_message>
<xml_diff>
--- a/data/leakdata.xlsx
+++ b/data/leakdata.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -498,37 +498,37 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>The confidential file was accessed using Ethan's credentials.</t>
+          <t>An anonymous tip claimed Ethan bragged about the leak in a private chat.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Authentication proves which account was active, not who was physically using the workstation.</t>
+          <t>A screenshot circulated online showing a chat message attributed to Ethan admitting to the leak.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>IT confirms lab workstations only auto-lock after 30 minutes of total inactivity.</t>
+          <t>Metadata on the screenshot shows it was created and edited after the leak had already gone viral.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>The folder access happened just 8 minutes into that window, well inside the no-relock period.</t>
+          <t>The account named in the screenshot does not match any of Ethan's real usernames, the message was fabricated.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>True, but incomplete</t>
+          <t>False / Fabricated</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High / Red Herring</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>F2, H1</t>
+          <t>E4, H3</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -545,37 +545,37 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Loading-dock footage shows someone resembling Noah returning to the building.</t>
+          <t>A temporary storage device found among a contractor's belongings contains traces of the Helix file structure.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Clothing and build are consistent with Noah, but the face is only partially visible.</t>
+          <t>File timestamps are consistent with the period immediately before the 11:47 PM upload.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>The figure carries a bag similar in size and shape to one later found among Noah's belongings.</t>
+          <t>The device shows the Helix demo file copied at 11:41 PM, then deleted from the device at 11:48 PM.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Combined with the exit-then-reentry pattern, this places someone matching Noah back inside minutes before the badge was used.</t>
+          <t>Records tie the device to Noah, and the copy-then-delete pattern matches someone erasing their tracks right after uploading.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Supporting, not conclusive alone</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>E2, H3</t>
+          <t>F2, D3</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -592,22 +592,22 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>A colleague on the call noticed Ethan's badge was missing from his lanyard clip before the meeting even started.</t>
+          <t>Ethan was visibly present on the video call.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>A coworker recalls glancing at Ethan's lanyard during the meeting and not seeing his badge clipped to it.</t>
+          <t>Multiple participants confirm seeing and speaking with him during the period when Lab 3 was accessed.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>This matches the timeline of when Ethan says he left it behind in Lab 3.</t>
+          <t>Two separate colleagues recall Ethan answering a direct question at 11:38 PM, one minute before the folder was accessed.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>It places the badge's disappearance before 11:24 PM, consistent with Noah having the opportunity to take it early.</t>
+          <t>It is not physically possible to be speaking on camera and typing in Lab 3 at the same instant.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -617,12 +617,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>B2, H3</t>
+          <t>B2, E1, C3</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -639,27 +639,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>The additional unsafe-response clip appears to be part of Project Helix.</t>
+          <t>A second version of the leaked video appeared online at 11:54 PM.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>The clip does not exist anywhere in the original internal demo.</t>
+          <t>The second file contains an additional segment not present in the original upload.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Engineers who ran the original demo confirm the model never produced that response in any recorded session.</t>
+          <t>The added segment runs 47 seconds and shows a fabricated 'unsafe response' clip.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>The clip was created separately and spliced in, it did not come from Project Helix at all.</t>
+          <t>Someone had access to the original leaked file and editing tools within those seven minutes.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>False / Manipulated</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>G2, A2</t>
+          <t>D3, G4</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>G1, D4, B2</t>
+          <t>B2, G1</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -733,22 +733,22 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Avery flagged unusual login patterns days before the leak, but was told the issue was low priority.</t>
+          <t>The security engineer was the one who discovered the leak had occurred and escalated it immediately.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>An internal ticket shows Avery reported suspicious badge-sharing behavior three days before the incident.</t>
+          <t>Server monitoring alerts show Avery's account was first to flag anomalous outbound traffic at 11:49 PM.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Management marked the ticket 'low priority, revisit next quarter.'</t>
+          <t>She escalated to her manager within two minutes of the alert, well before the video went viral.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>The exact vulnerability she flagged, a badge used without its owner present, is what let the leak happen.</t>
+          <t>Someone trying to cover their tracks is not usually the one who raises the alarm.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F2, H4</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -780,27 +780,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Security footage shows a person in a dark hoodie entering the Lab 3 hallway at 11:33 PM.</t>
+          <t>Ethan later reported that his badge had been missing.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>The person's face is never clearly visible. Identity was inferred partly from clothing.</t>
+          <t>Ethan last remembers having it before leaving Lab 3 earlier that evening.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>The company issues the same style of dark hoodie to every employee at onboarding.</t>
+          <t>He reported it missing to Avery's team at 11:56 PM, nine minutes after the leak.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>At least three of the four suspects own an identical hoodie, per the merchandise order records.</t>
+          <t>He reported it before he had any way of knowing a leak had even happened.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>True, but incomplete</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>E1, B2, H3</t>
+          <t>E1, A4</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -827,42 +827,38 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>The Lab 3 workstation remained logged into Ethan's account after Ethan left.</t>
+          <t>A rumor circulated that someone had been secretly recording internal meetings for weeks.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Someone could access Project Helix without knowing Ethan's password.</t>
+          <t>Two employees mention hearing this rumor in the days before the leak.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>The workstation's session timeout is set to 60 minutes, unusually long for a machine handling confidential files.</t>
+          <t>Neither can say where the rumor started.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>That single configuration gap is what turned a forgotten badge into a full breach.</t>
+          <t>Security finds no evidence any meeting was ever recorded without consent.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Unsubstantiated rumor</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>F2, A1, H3</t>
-        </is>
-      </c>
+          <t>Low / Red Herring</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Noah</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -874,22 +870,22 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>The second video uses different encoding settings from the first.</t>
+          <t>The Lab 3 workstation remained logged into Ethan's account after Ethan left.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Metadata suggests the additional segment was edited on a different device shortly before 11:54 PM.</t>
+          <t>Someone could access Project Helix without knowing Ethan's password.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>The encoding profile matches a specific video editing application, not the format used for internal demo recordings.</t>
+          <t>The workstation's session timeout is set to 60 minutes, unusually long for a machine handling confidential files.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>That application is installed on exactly one company device.</t>
+          <t>That single configuration gap is what turned a forgotten badge into a full breach.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -904,12 +900,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>D1, B4</t>
+          <t>C3, E05, A4</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Olivia</t>
+          <t>Noah</t>
         </is>
       </c>
     </row>
@@ -921,22 +917,22 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Ethan later reported that his badge had been missing.</t>
+          <t>Ethan says he was on a video call during the incident.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Ethan last remembers having it before leaving Lab 3 earlier that evening.</t>
+          <t>Meeting records show Ethan joined at 11:24 PM and remained connected until about 11:53 PM.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>He reported it missing to Avery's team at 11:56 PM, nine minutes after the leak.</t>
+          <t>The call platform logs an unbroken connection, no drops and no rejoins, for the full 29 minutes.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>He reported it before he had any way of knowing a leak had even happened.</t>
+          <t>That window fully covers the badge swipe, the folder access, and the upload.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -946,12 +942,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>E1, H3</t>
+          <t>E1, C1</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -968,42 +964,42 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Avery had administrator access to almost every system involved.</t>
+          <t>Olivia's laptop contains the editing environment consistent with the altered video.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>No logs show Avery using privileged access during the relevant period.</t>
+          <t>Software activity shows editing shortly before the second upload.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Her admin credentials were not used to touch any Helix-related file, folder, or system that night.</t>
+          <t>The application's autosave history shows a project file opened at 11:44 PM and exported at 11:53 PM.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Having the keys to every door is not evidence of walking through one.</t>
+          <t>That is the exact editing application and window identified in the encoding metadata.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>True, but low relevance</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Low / Red Herring</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>F3, G4</t>
+          <t>E3, B4</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Avery</t>
+          <t>Olivia</t>
         </is>
       </c>
     </row>
@@ -1015,42 +1011,42 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Ethan opposed the Project Helix launch and wanted it delayed.</t>
+          <t>The security engineer's own system logs are the most complete record of the night, since she personally maintains the logging infrastructure.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Internal messages show Ethan repeatedly raised safety concerns about releasing the model too early.</t>
+          <t>As the security engineer, Avery configured and maintains every log referenced in this investigation.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>He proposed delaying the launch by at least two weeks, in a message sent to the whole leadership team.</t>
+          <t>That gives her more technical opportunity than anyone else in the building.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Leadership rejected the delay in writing, giving Ethan a documented but overruled grievance.</t>
+          <t>But the (independently cross-checked) logs show no tampering or gaps around her own account.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>True, but motive alone proves nothing</t>
+          <t>True, but shows opportunity, not guilt</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Medium / Red Herring</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>D4, E3, C3</t>
+          <t>F3, H4</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>Avery</t>
         </is>
       </c>
     </row>
@@ -1062,42 +1058,38 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Noah's contractor badge indicates that he had already left the building.</t>
+          <t>A one-day visitor badge was issued earlier that day to an outside vendor unrelated to the four people still in the building.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>His own badge was used to exit, but a loading-dock camera suggests he later re-entered behind another employee.</t>
+          <t>Front desk logs show the visitor badge was issued at 2 PM for a scheduled equipment demo.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>The exit swipe was logged at 9:58 PM, over an hour before the leak.</t>
+          <t>The visitor signed out at 5:30 PM, well before the incident window began.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>An exit swipe only proves he left once, it says nothing about whether he came back.</t>
+          <t>Their badge was deactivated at sign-out and was never used again that night.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>True record, misleading conclusion</t>
+          <t>TRUE, but irrelevant</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>H3, B1</t>
-        </is>
-      </c>
+          <t>Low / Red Herring</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Noah</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1109,27 +1101,27 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Ethan's account accessed the confidential Project Helix folder at 11:39 PM.</t>
+          <t>The original leaked video was uploaded at 11:47 PM from Lab 3's network.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>No new password was entered. The workstation had already been logged into Ethan's account.</t>
+          <t>Network records identify the location of the connection, not the individual using it.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>The session had begun over an hour earlier, before Ethan left for his call.</t>
+          <t>Lab 3's Wi-Fi range extends into the adjacent break room and stairwell, neither of which needs a badge.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Anyone sitting down at that terminal would have had full access without ever needing his password.</t>
+          <t>The upload could have originated from anyone in that wider radius, not only someone inside the locked lab.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>True, but misleading</t>
+          <t>True, but incomplete</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1139,7 +1131,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>A1, H1</t>
+          <t>C3, B1</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1156,42 +1148,42 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>A second version of the leaked video appeared online at 11:54 PM.</t>
+          <t>Loading-dock footage shows someone resembling Noah returning to the building.</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>The second file contains an additional segment not present in the original upload.</t>
+          <t>Clothing and build are consistent with Noah, but the face is only partially visible.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>The added segment runs 47 seconds and shows a fabricated 'unsafe response' clip.</t>
+          <t>The figure carries a bag similar in size and shape to one later found among Noah's belongings.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Someone had access to the original leaked file and editing tools within those seven minutes.</t>
+          <t>Combined with the exit-then-reentry pattern, this places someone matching Noah back inside minutes before the badge was used.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Supporting, not conclusive alone</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>B3, D1</t>
+          <t>F4, A4</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Olivia</t>
+          <t>Noah</t>
         </is>
       </c>
     </row>
@@ -1203,42 +1195,42 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Ethan's badge, account, and network location all independently point to Ethan.</t>
+          <t>The product lead strongly wanted the launch to continue.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>All three signals could result from one person using Ethan's badge and already-authenticated workstation inside Lab 3.</t>
+          <t>Internal messages show she feared a delay would jeopardize a major launch and partnership.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Security consultants confirm this exact scenario, badge theft plus an unlocked terminal, has happened before elsewhere.</t>
+          <t>She wrote that a delay 'could cost us the partnership entirely,' three days before the leak.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Three suspicious signals near the same name is not the same thing as three independent proofs.</t>
+          <t>Discrediting the leak, not stopping it, would have been enough to save the launch.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>False combined inference</t>
+          <t>True / Motive</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>E1, F2, A4</t>
+          <t>C2, B4</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>Olivia</t>
         </is>
       </c>
     </row>
@@ -1250,37 +1242,37 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Avery's system logs are the most complete record of the night, since she personally maintains the logging infrastructure.</t>
+          <t>Avery's badge and login activity that night were both located at her desk on a different floor.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>As the security engineer, Avery configured and maintains every log referenced in this investigation.</t>
+          <t>Badge logs show Avery working from her own desk on the third floor from 10 PM until after midnight.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>That gives her more technical opportunity than anyone else in the building.</t>
+          <t>Her login sessions during that window match routine end-of-day security patch work, unrelated to Lab 3 or Helix.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>But the (independently cross-checked) logs show no tampering or gaps around her own account.</t>
+          <t>None of her recorded activity overlaps with the Lab 3 access window at all.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>True, but shows opportunity, not guilt</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>C2, F3</t>
+          <t>F3, H4</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1297,42 +1289,38 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>The first leaked video matches the internal Helix demo.</t>
+          <t>The building's thermostat logged an unusual temperature drop in Lab 3 around midnight.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>File comparison shows no added clips or major modification before the first upload.</t>
+          <t>Facilities data shows the room cooled by four degrees starting at 11:40 PM.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Even compression artifacts and audio levels match the internal master file in the unedited sections.</t>
+          <t>Maintenance says this matches a routine HVAC cycle that runs every night at that time.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Whoever uploaded the first video did not alter it, they only moved it.</t>
+          <t>The timing is coincidental and unrelated to anyone's presence.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Coincidence</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>E4, G2</t>
-        </is>
-      </c>
+          <t>Low / Red Herring</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Noah</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1344,37 +1332,37 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>An anonymous tip claimed Ethan bragged about the leak in a private chat.</t>
+          <t>Ethan's account accessed the confidential Project Helix folder at 11:39 PM.</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>A screenshot circulated online showing a chat message attributed to Ethan admitting to the leak.</t>
+          <t>No new password was entered. The workstation had already been logged into Ethan's account.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Metadata on the screenshot shows it was created and edited after the leak had already gone viral.</t>
+          <t>The session had begun over an hour earlier, before Ethan left for his call.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>The account named in the screenshot does not match any of Ethan's real usernames, the message was fabricated.</t>
+          <t>Anyone sitting down at that terminal would have had full access without ever needing his password.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>False / Fabricated</t>
+          <t>True, but misleading</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>High / Red Herring</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>H2, D2</t>
+          <t>F2, A2</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1391,22 +1379,22 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Olivia's device connected to an external file-sharing service shortly before 11:54 PM.</t>
+          <t>The first leaked video matches the internal Helix demo.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>The connection timing is consistent with the second upload, not the original 11:47 upload.</t>
+          <t>File comparison shows no added clips or major modification before the first upload.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>The outbound connection at 11:54 PM matches the same file-sharing service, down to the session ID range.</t>
+          <t>Even compression artifacts and audio levels match the internal master file in the unedited sections.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Olivia's device was actively uploading at the exact minute the second video appeared.</t>
+          <t>Whoever uploaded the first video did not alter it, they only moved it.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1421,12 +1409,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>G2, B4</t>
+          <t>B1, D1</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Olivia</t>
+          <t>Noah</t>
         </is>
       </c>
     </row>
@@ -1438,22 +1426,22 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Ethan was visibly present on the video call.</t>
+          <t>The second video uses different encoding settings from the first.</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Multiple participants confirm seeing and speaking with him during the period when Lab 3 was accessed.</t>
+          <t>Metadata suggests the additional segment was edited on a different device shortly before 11:54 PM.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Two separate colleagues recall Ethan answering a direct question at 11:38 PM, one minute before the folder was accessed.</t>
+          <t>The encoding profile matches a specific video editing application, not the format used for internal demo recordings.</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>It is not physically possible to be speaking on camera and typing in Lab 3 at the same instant.</t>
+          <t>That application is installed on exactly one company device.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1468,12 +1456,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>D4, E1, F2</t>
+          <t>G4, C2</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>Olivia</t>
         </is>
       </c>
     </row>
@@ -1485,37 +1473,37 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Avery previously warned that the building's identity and access systems were insecure.</t>
+          <t>The security engineer had administrator access to almost every system involved.</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Her warnings specifically mention badge sharing and unattended authenticated workstations.</t>
+          <t>No logs show Avery using privileged access during the relevant period.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>She filed that warning eleven days before the leak, describing this exact scenario almost precisely.</t>
+          <t>Her admin credentials were not used to touch any Helix-related file, folder, or system that night.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>The vulnerability she predicted is the one that was actually used, just not by her.</t>
+          <t>Having the keys to every door is not evidence of walking through one.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>True and relevant context</t>
+          <t>True, but low relevance</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low / Red Herring</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>E1, H1</t>
+          <t>H4, A3</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1532,42 +1520,38 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Ethan's laptop was still connected to the video call's screen-share the entire time Lab 3 was accessed.</t>
+          <t>An unrelated security incident from six months ago turned up in the same server logs.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Screen-share logs show continuous activity from Ethan's laptop throughout the window in question.</t>
+          <t>The log viewer surfaces an entry from an old badge-cloning incident, unconnected to Project Helix.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>The shared screen displayed a slide deck Ethan was actively presenting, timestamped every few seconds.</t>
+          <t>That earlier incident was already resolved, and the employee involved no longer works at the company.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>It would have been physically impossible for Ethan to present live on the call and be in Lab 3 at the same time.</t>
+          <t>It only appears in this report because the logging system wasn't filtered by date.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Unrelated, resolved</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>D4, E3</t>
-        </is>
-      </c>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1579,42 +1563,42 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Noah was near Ethan's belongings before the unauthorized Lab 3 entry.</t>
+          <t>The lead researcher opposed the Project Helix launch and wanted it delayed.</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Noah had an opportunity to take Ethan's badge before 11:31 PM.</t>
+          <t>Internal messages show Ethan repeatedly raised safety concerns about releasing the model too early.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Noah was seen near the jacket rack by the lab entrance at 11:22 PM, six minutes after Ethan left it there.</t>
+          <t>He proposed delaying the launch by at least two weeks, in a message sent to the whole leadership team.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>No one else is placed near that rack in the eleven minutes before the badge was used.</t>
+          <t>Leadership rejected the delay in writing, giving Ethan a documented but overruled grievance.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True, but motive alone proves nothing</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium / Red Herring</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>E1, B2, E4</t>
+          <t>B2, C1, A1</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Noah</t>
+          <t>Ethan</t>
         </is>
       </c>
     </row>
@@ -1626,42 +1610,42 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>The original leaked video was uploaded at 11:47 PM from Lab 3's network.</t>
+          <t>Noah was near Ethan's belongings before the unauthorized Lab 3 entry.</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Network records identify the location of the connection, not the individual using it.</t>
+          <t>Noah had an opportunity to take Ethan's badge before 11:31 PM.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Lab 3's Wi-Fi range extends into the adjacent break room and stairwell, neither of which needs a badge.</t>
+          <t>Noah was seen near the jacket rack by the lab entrance at 11:22 PM, six minutes after Ethan left it there.</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>The upload could have originated from anyone in that wider radius, not only someone inside the locked lab.</t>
+          <t>No one else is placed near that rack in the eleven minutes before the badge was used.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>True, but incomplete</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>F2, E4</t>
+          <t>E1, G1, B1</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>Noah</t>
         </is>
       </c>
     </row>
@@ -1673,22 +1657,22 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Olivia's laptop contains the editing environment consistent with the altered video.</t>
+          <t>Olivia's device connected to an external file-sharing service shortly before 11:54 PM.</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Software activity shows editing shortly before the second upload.</t>
+          <t>The connection timing is consistent with the second upload, not the original 11:47 upload.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>The application's autosave history shows a project file opened at 11:44 PM and exported at 11:53 PM.</t>
+          <t>The outbound connection at 11:54 PM matches the same file-sharing service, down to the session ID range.</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>That is the exact editing application and window identified in the encoding metadata.</t>
+          <t>Olivia's device was actively uploading at the exact minute the second video appeared.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1703,7 +1687,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>A2, D3</t>
+          <t>D1, C2</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -1720,22 +1704,22 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Avery was the one who discovered the leak had occurred and escalated it immediately.</t>
+          <t>The security engineer flagged unusual login patterns days before the leak, but was told the issue was low priority.</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Server monitoring alerts show Avery's account was first to flag anomalous outbound traffic at 11:49 PM.</t>
+          <t>An internal ticket shows Avery reported suspicious badge-sharing behavior three days before the incident.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>She escalated to her manager within two minutes of the alert, well before the video went viral.</t>
+          <t>Management marked the ticket 'low priority, revisit next quarter.'</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Someone trying to cover their tracks is not usually the one who raises the alarm.</t>
+          <t>The exact vulnerability she flagged, a badge used without its owner present, is what let the leak happen.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1750,7 +1734,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>A4, F3</t>
+          <t>H4</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -1767,27 +1751,27 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Ethan says he was on a video call during the incident.</t>
+          <t>The two leaked videos probably came from the same person because they appeared seven minutes apart.</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Meeting records show Ethan joined at 11:24 PM and remained connected until about 11:53 PM.</t>
+          <t>File structure, editing metadata, and upload behavior indicate two separate actions.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>The call platform logs an unbroken connection, no drops and no rejoins, for the full 29 minutes.</t>
+          <t>The two uploads used different devices and different accounts.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>That window fully covers the badge swipe, the folder access, and the upload.</t>
+          <t>Two people made two separate decisions, seven minutes apart, for two different reasons.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>False assumption</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -1797,12 +1781,12 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>E1, E3</t>
+          <t>D3, D1, E3</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1814,27 +1798,27 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>A temporary storage device associated with Noah contains traces of the Helix file structure.</t>
+          <t>Ethan's badge, account, and network location all independently point to Ethan.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>File timestamps are consistent with the period immediately before the 11:47 PM upload.</t>
+          <t>All three signals could result from one person using Ethan's badge and already-authenticated workstation inside Lab 3.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>The device shows the Helix demo file copied at 11:41 PM, then deleted from the device at 11:48 PM.</t>
+          <t>Security consultants confirm this exact scenario, badge theft plus an unlocked terminal, has happened before elsewhere.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>That copy-then-delete pattern matches someone erasing their tracks right after uploading.</t>
+          <t>Three suspicious signals near the same name is not the same thing as three independent proofs.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>False combined inference</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1844,12 +1828,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>A4, B3</t>
+          <t>E1, C3, F2</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Noah</t>
+          <t>Ethan</t>
         </is>
       </c>
     </row>
@@ -1861,42 +1845,42 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Olivia strongly wanted the product launch to continue.</t>
+          <t>The contractor's badge indicates that he had already left the building.</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Internal messages show she feared a delay would jeopardize a major launch and partnership.</t>
+          <t>His own badge was used to exit, but a loading-dock camera suggests he later re-entered behind another employee.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>She wrote that a delay 'could cost us the partnership entirely,' three days before the leak.</t>
+          <t>The exit swipe was logged at 9:58 PM, over an hour before the leak.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Discrediting the leak, not stopping it, would have been enough to save the launch.</t>
+          <t>An exit swipe only proves he left once, it says nothing about whether he came back.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>True / Motive</t>
+          <t>True record, misleading conclusion</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>B4, D3</t>
+          <t>A4, G2</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Olivia</t>
+          <t>Noah</t>
         </is>
       </c>
     </row>
@@ -1908,42 +1892,42 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Avery's badge and login activity that night were both located at her desk on a different floor.</t>
+          <t>The additional unsafe-response clip appears to be part of Project Helix.</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Badge logs show Avery working from her own desk on the third floor from 10 PM until after midnight.</t>
+          <t>The clip does not exist anywhere in the original internal demo.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Her login sessions during that window match routine end-of-day security patch work, unrelated to Lab 3 or Helix.</t>
+          <t>Engineers who ran the original demo confirm the model never produced that response in any recorded session.</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>None of her recorded activity overlaps with the Lab 3 access window at all.</t>
+          <t>The clip was created separately and spliced in, it did not come from Project Helix at all.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>False / Manipulated</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>C2, F3</t>
+          <t>D1, E3</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Avery</t>
+          <t>Olivia</t>
         </is>
       </c>
     </row>
@@ -1955,40 +1939,83 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>The two leaked videos probably came from the same person because they appeared seven minutes apart.</t>
+          <t>The security engineer previously warned that the building's identity and access systems were insecure.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>File structure, editing metadata, and upload behavior indicate two separate actions.</t>
+          <t>Her warnings specifically mention badge sharing and unattended authenticated workstations.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>The two uploads used different devices and different accounts.</t>
+          <t>She filed that warning eleven days before the leak, describing this exact scenario almost precisely.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Two people made two separate decisions, seven minutes apart, for two different reasons.</t>
+          <t>The vulnerability she predicted is the one that was actually used, just not by her.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>False assumption</t>
+          <t>True and relevant context</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>B3, G2, A2</t>
+          <t>E1, A2</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Avery</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Someone ordered late-night food delivery to the building's side entrance at 11:15 PM.</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>A delivery service confirms a drop-off at the side entrance twenty minutes before the badge swipe.</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Building logs show the side entrance door was propped open for about six minutes around that delivery.</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>No badge or camera record identifies who received the delivery.</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Unverified, no clear connection</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2005,7 +2032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2028,170 +2055,184 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ethan (E05-&gt;A1)</t>
+          <t>Ethan (A1)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Noah (E16-&gt;B1)</t>
+          <t>Noah (B1)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ethan (E27-&gt;C1)</t>
+          <t>Ethan (C1)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Olivia (E18-&gt;D1)</t>
+          <t>Olivia (D1)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Ethan (E02-&gt;E1)</t>
+          <t>Ethan (E1)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Avery (E29-&gt;F1)</t>
+          <t>Avery (F1)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Ethan (E03-&gt;G1)</t>
+          <t>Ethan (G1)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Noah (E12-&gt;H1)</t>
+          <t>— (H1)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Olivia (E19-&gt;A2)</t>
+          <t>Noah (A2)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ethan (E10-&gt;B2)</t>
+          <t>Ethan (B2)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Avery (E23-&gt;C2)</t>
+          <t>Olivia (C2)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ethan (E01-&gt;D2)</t>
+          <t>Avery (D2)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Noah (E15-&gt;E2)</t>
+          <t>— (E2)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Ethan (E04-&gt;F2)</t>
+          <t>Ethan (F2)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Olivia (E17-&gt;G2)</t>
+          <t>Noah (G2)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Ethan (E07-&gt;H2)</t>
+          <t>Olivia (H2)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Avery (E31-&gt;A3)</t>
+          <t>Avery (A3)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Noah (E14-&gt;B3)</t>
+          <t>— (B3)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ethan (E32-&gt;C3)</t>
+          <t>Ethan (C3)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Olivia (E21-&gt;D3)</t>
+          <t>Noah (D3)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Ethan (E09-&gt;E3)</t>
+          <t>Olivia (E3)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Avery (E24-&gt;F3)</t>
+          <t>Avery (F3)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Ethan (E26-&gt;G3)</t>
+          <t>— (G3)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Noah (E11-&gt;H3)</t>
+          <t>Ethan (H3)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ethan (E06-&gt;A4)</t>
+          <t>Noah (A4)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Olivia (E20-&gt;B4)</t>
+          <t>Olivia (B4)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Avery (E30-&gt;C4)</t>
+          <t>Avery (C4)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ethan (E08-&gt;D4)</t>
+          <t>— (D4)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Noah (E13-&gt;E4)</t>
+          <t>Ethan (E4)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Olivia (E22-&gt;F4)</t>
+          <t>Noah (F4)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Avery (E28-&gt;G4)</t>
+          <t>Olivia (G4)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>— (E25-&gt;H4)</t>
-        </is>
-      </c>
+          <t>Avery (H4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>— (A5)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2204,7 +2245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2236,11 +2277,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>D4, E3, B2, G3, C1</t>
+          <t>B2, C1, G1</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2296,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>H3, H1, E4, B3, B1</t>
+          <t>A4, A2, B1, D3, G2</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2311,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>G2, A2, B4, D3, F4</t>
+          <t>D1, E3, C2, B4, H2</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2326,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>F3, G4, F1, C4, A3</t>
+          <t>H4, A3, C4, F1, D2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Dropped: E03 (redundant with E02's badge point), E05 (redundant with E04), E26/E27 (redundant extra alibi pieces).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deal onto two ranks top and bottom, 32 pieces, middle board clear
Board now looks like a real opening position: evidence sits on ranks
1-2 and 7-8 (16 squares each), ranks 3-6 stay empty, instead of one
contiguous block filling the top of the board. Dropped one noise item
(the food-delivery red herring) to land on exactly 32 = 2 rows x 8
cols x 2 blocks. Re-ran the anti-clustering scheduler so no two board
neighbours (including across the two blocks' own internal rows) point
at the same suspect, and fixed a stray dangling connects-to reference
(E12 pointed at the already-removed E05).
</commit_message>
<xml_diff>
--- a/data/leakdata.xlsx
+++ b/data/leakdata.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -498,37 +498,37 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>An anonymous tip claimed Ethan bragged about the leak in a private chat.</t>
+          <t>The lead researcher opposed the Project Helix launch and wanted it delayed.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>A screenshot circulated online showing a chat message attributed to Ethan admitting to the leak.</t>
+          <t>Internal messages show Ethan repeatedly raised safety concerns about releasing the model too early.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Metadata on the screenshot shows it was created and edited after the leak had already gone viral.</t>
+          <t>He proposed delaying the launch by at least two weeks, in a message sent to the whole leadership team.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>The account named in the screenshot does not match any of Ethan's real usernames, the message was fabricated.</t>
+          <t>Leadership rejected the delay in writing, giving Ethan a documented but overruled grievance.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>False / Fabricated</t>
+          <t>True, but motive alone proves nothing</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>High / Red Herring</t>
+          <t>Medium / Red Herring</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>E4, H3</t>
+          <t>B7, F2, B2</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -545,22 +545,22 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>A temporary storage device found among a contractor's belongings contains traces of the Helix file structure.</t>
+          <t>Noah was near Ethan's belongings before the unauthorized Lab 3 entry.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>File timestamps are consistent with the period immediately before the 11:47 PM upload.</t>
+          <t>Noah had an opportunity to take Ethan's badge before 11:31 PM.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>The device shows the Helix demo file copied at 11:41 PM, then deleted from the device at 11:48 PM.</t>
+          <t>Noah was seen near the jacket rack by the lab entrance at 11:22 PM, six minutes after Ethan left it there.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Records tie the device to Noah, and the copy-then-delete pattern matches someone erasing their tracks right after uploading.</t>
+          <t>No one else is placed near that rack in the eleven minutes before the badge was used.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -570,12 +570,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>F2, D3</t>
+          <t>C1, G1, H1</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -592,27 +592,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Ethan was visibly present on the video call.</t>
+          <t>Ethan's badge entered Lab 3 at 11:31 PM.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Multiple participants confirm seeing and speaking with him during the period when Lab 3 was accessed.</t>
+          <t>The access system records the credential used, not the identity of the person carrying it.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Two separate colleagues recall Ethan answering a direct question at 11:38 PM, one minute before the folder was accessed.</t>
+          <t>Facilities confirms badge readers have no camera or biometric check attached to them.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>It is not physically possible to be speaking on camera and typing in Lab 3 at the same instant.</t>
+          <t>The log entry only proves the badge was there, not that Ethan was.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True, but misleading</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>B2, E1, C3</t>
+          <t>B7, G1</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -639,22 +639,22 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>A second version of the leaked video appeared online at 11:54 PM.</t>
+          <t>The second video uses different encoding settings from the first.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>The second file contains an additional segment not present in the original upload.</t>
+          <t>Metadata suggests the additional segment was edited on a different device shortly before 11:54 PM.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>The added segment runs 47 seconds and shows a fabricated 'unsafe response' clip.</t>
+          <t>The encoding profile matches a specific video editing application, not the format used for internal demo recordings.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Someone had access to the original leaked file and editing tools within those seven minutes.</t>
+          <t>That application is installed on exactly one company device.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>D3, G4</t>
+          <t>G2, A2</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -686,27 +686,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Ethan's badge entered Lab 3 at 11:31 PM.</t>
+          <t>The original leaked video was uploaded at 11:47 PM from Lab 3's network.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>The access system records the credential used, not the identity of the person carrying it.</t>
+          <t>Network records identify the location of the connection, not the individual using it.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Facilities confirms badge readers have no camera or biometric check attached to them.</t>
+          <t>Lab 3's Wi-Fi range extends into the adjacent break room and stairwell, neither of which needs a badge.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>The log entry only proves the badge was there, not that Ethan was.</t>
+          <t>The upload could have originated from anyone in that wider radius, not only someone inside the locked lab.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>True, but misleading</t>
+          <t>True, but incomplete</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>B2, G1</t>
+          <t>G7, H1</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -733,37 +733,37 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>The security engineer was the one who discovered the leak had occurred and escalated it immediately.</t>
+          <t>The security engineer had administrator access to almost every system involved.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Server monitoring alerts show Avery's account was first to flag anomalous outbound traffic at 11:49 PM.</t>
+          <t>No logs show Avery using privileged access during the relevant period.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>She escalated to her manager within two minutes of the alert, well before the video went viral.</t>
+          <t>Her admin credentials were not used to touch any Helix-related file, folder, or system that night.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Someone trying to cover their tracks is not usually the one who raises the alarm.</t>
+          <t>Having the keys to every door is not evidence of walking through one.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True, but low relevance</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low / Red Herring</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>F2, H4</t>
+          <t>C2, G8</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>E1, A4</t>
+          <t>C1, B1</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -827,38 +827,42 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>A rumor circulated that someone had been secretly recording internal meetings for weeks.</t>
+          <t>A temporary storage device found among a contractor's belongings contains traces of the Helix file structure.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Two employees mention hearing this rumor in the days before the leak.</t>
+          <t>File timestamps are consistent with the period immediately before the 11:47 PM upload.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Neither can say where the rumor started.</t>
+          <t>The device shows the Helix demo file copied at 11:41 PM, then deleted from the device at 11:48 PM.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Security finds no evidence any meeting was ever recorded without consent.</t>
+          <t>Records tie the device to Noah, and the copy-then-delete pattern matches someone erasing their tracks right after uploading.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Unsubstantiated rumor</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Low / Red Herring</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr"/>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>E1, H7</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Noah</t>
         </is>
       </c>
     </row>
@@ -870,22 +874,22 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>The Lab 3 workstation remained logged into Ethan's account after Ethan left.</t>
+          <t>Olivia's laptop contains the editing environment consistent with the altered video.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Someone could access Project Helix without knowing Ethan's password.</t>
+          <t>Software activity shows editing shortly before the second upload.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>The workstation's session timeout is set to 60 minutes, unusually long for a machine handling confidential files.</t>
+          <t>The application's autosave history shows a project file opened at 11:44 PM and exported at 11:53 PM.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>That single configuration gap is what turned a forgotten badge into a full breach.</t>
+          <t>That is the exact editing application and window identified in the encoding metadata.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -900,12 +904,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>C3, E05, A4</t>
+          <t>D1, D7</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Noah</t>
+          <t>Olivia</t>
         </is>
       </c>
     </row>
@@ -917,37 +921,37 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Ethan says he was on a video call during the incident.</t>
+          <t>An anonymous tip claimed Ethan bragged about the leak in a private chat.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Meeting records show Ethan joined at 11:24 PM and remained connected until about 11:53 PM.</t>
+          <t>A screenshot circulated online showing a chat message attributed to Ethan admitting to the leak.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>The call platform logs an unbroken connection, no drops and no rejoins, for the full 29 minutes.</t>
+          <t>Metadata on the screenshot shows it was created and edited after the leak had already gone viral.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>That window fully covers the badge swipe, the folder access, and the upload.</t>
+          <t>The account named in the screenshot does not match any of Ethan's real usernames, the message was fabricated.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>False / Fabricated</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High / Red Herring</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>E1, C1</t>
+          <t>D8, A1</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -964,42 +968,42 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Olivia's laptop contains the editing environment consistent with the altered video.</t>
+          <t>The security engineer previously warned that the building's identity and access systems were insecure.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Software activity shows editing shortly before the second upload.</t>
+          <t>Her warnings specifically mention badge sharing and unattended authenticated workstations.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>The application's autosave history shows a project file opened at 11:44 PM and exported at 11:53 PM.</t>
+          <t>She filed that warning eleven days before the leak, describing this exact scenario almost precisely.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>That is the exact editing application and window identified in the encoding metadata.</t>
+          <t>The vulnerability she predicted is the one that was actually used, just not by her.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True and relevant context</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>E3, B4</t>
+          <t>C1, E8</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Olivia</t>
+          <t>Avery</t>
         </is>
       </c>
     </row>
@@ -1011,42 +1015,38 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>The security engineer's own system logs are the most complete record of the night, since she personally maintains the logging infrastructure.</t>
+          <t>The building's thermostat logged an unusual temperature drop in Lab 3 around midnight.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>As the security engineer, Avery configured and maintains every log referenced in this investigation.</t>
+          <t>Facilities data shows the room cooled by four degrees starting at 11:40 PM.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>That gives her more technical opportunity than anyone else in the building.</t>
+          <t>Maintenance says this matches a routine HVAC cycle that runs every night at that time.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>But the (independently cross-checked) logs show no tampering or gaps around her own account.</t>
+          <t>The timing is coincidental and unrelated to anyone's presence.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>True, but shows opportunity, not guilt</t>
+          <t>Coincidence</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>F3, H4</t>
-        </is>
-      </c>
+          <t>Low / Red Herring</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Avery</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1058,38 +1058,42 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>A one-day visitor badge was issued earlier that day to an outside vendor unrelated to the four people still in the building.</t>
+          <t>The contractor's badge indicates that he had already left the building.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Front desk logs show the visitor badge was issued at 2 PM for a scheduled equipment demo.</t>
+          <t>His own badge was used to exit, but a loading-dock camera suggests he later re-entered behind another employee.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>The visitor signed out at 5:30 PM, well before the incident window began.</t>
+          <t>The exit swipe was logged at 9:58 PM, over an hour before the leak.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Their badge was deactivated at sign-out and was never used again that night.</t>
+          <t>An exit swipe only proves he left once, it says nothing about whether he came back.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>TRUE, but irrelevant</t>
+          <t>True record, misleading conclusion</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Low / Red Herring</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>B1, C7</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Noah</t>
         </is>
       </c>
     </row>
@@ -1101,27 +1105,27 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>The original leaked video was uploaded at 11:47 PM from Lab 3's network.</t>
+          <t>Ethan was visibly present on the video call.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Network records identify the location of the connection, not the individual using it.</t>
+          <t>Multiple participants confirm seeing and speaking with him during the period when Lab 3 was accessed.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Lab 3's Wi-Fi range extends into the adjacent break room and stairwell, neither of which needs a badge.</t>
+          <t>Two separate colleagues recall Ethan answering a direct question at 11:38 PM, one minute before the folder was accessed.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>The upload could have originated from anyone in that wider radius, not only someone inside the locked lab.</t>
+          <t>It is not physically possible to be speaking on camera and typing in Lab 3 at the same instant.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>True, but incomplete</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1131,7 +1135,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>C3, B1</t>
+          <t>B7, C1, G7</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1148,42 +1152,42 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Loading-dock footage shows someone resembling Noah returning to the building.</t>
+          <t>The additional unsafe-response clip appears to be part of Project Helix.</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Clothing and build are consistent with Noah, but the face is only partially visible.</t>
+          <t>The clip does not exist anywhere in the original internal demo.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>The figure carries a bag similar in size and shape to one later found among Noah's belongings.</t>
+          <t>Engineers who ran the original demo confirm the model never produced that response in any recorded session.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Combined with the exit-then-reentry pattern, this places someone matching Noah back inside minutes before the badge was used.</t>
+          <t>The clip was created separately and spliced in, it did not come from Project Helix at all.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Supporting, not conclusive alone</t>
+          <t>False / Manipulated</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>F4, A4</t>
+          <t>F8, D1</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Noah</t>
+          <t>Olivia</t>
         </is>
       </c>
     </row>
@@ -1195,27 +1199,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>The product lead strongly wanted the launch to continue.</t>
+          <t>The security engineer flagged unusual login patterns days before the leak, but was told the issue was low priority.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Internal messages show she feared a delay would jeopardize a major launch and partnership.</t>
+          <t>An internal ticket shows Avery reported suspicious badge-sharing behavior three days before the incident.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>She wrote that a delay 'could cost us the partnership entirely,' three days before the leak.</t>
+          <t>Management marked the ticket 'low priority, revisit next quarter.'</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Discrediting the leak, not stopping it, would have been enough to save the launch.</t>
+          <t>The exact vulnerability she flagged, a badge used without its owner present, is what let the leak happen.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>True / Motive</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1225,176 +1229,176 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>C2, B4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Olivia</t>
+          <t>Avery</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>A7</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Avery's badge and login activity that night were both located at her desk on a different floor.</t>
+          <t>A rumor circulated that someone had been secretly recording internal meetings for weeks.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Badge logs show Avery working from her own desk on the third floor from 10 PM until after midnight.</t>
+          <t>Two employees mention hearing this rumor in the days before the leak.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Her login sessions during that window match routine end-of-day security patch work, unrelated to Lab 3 or Helix.</t>
+          <t>Neither can say where the rumor started.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>None of her recorded activity overlaps with the Lab 3 access window at all.</t>
+          <t>Security finds no evidence any meeting was ever recorded without consent.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Unsubstantiated rumor</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>F3, H4</t>
-        </is>
-      </c>
+          <t>Low / Red Herring</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Avery</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>B7</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>The building's thermostat logged an unusual temperature drop in Lab 3 around midnight.</t>
+          <t>Ethan says he was on a video call during the incident.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Facilities data shows the room cooled by four degrees starting at 11:40 PM.</t>
+          <t>Meeting records show Ethan joined at 11:24 PM and remained connected until about 11:53 PM.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Maintenance says this matches a routine HVAC cycle that runs every night at that time.</t>
+          <t>The call platform logs an unbroken connection, no drops and no rejoins, for the full 29 minutes.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>The timing is coincidental and unrelated to anyone's presence.</t>
+          <t>That window fully covers the badge swipe, the folder access, and the upload.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Coincidence</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Low / Red Herring</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>C1, F2</t>
+        </is>
+      </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ethan</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Ethan's account accessed the confidential Project Helix folder at 11:39 PM.</t>
+          <t>Loading-dock footage shows someone resembling Noah returning to the building.</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>No new password was entered. The workstation had already been logged into Ethan's account.</t>
+          <t>Clothing and build are consistent with Noah, but the face is only partially visible.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>The session had begun over an hour earlier, before Ethan left for his call.</t>
+          <t>The figure carries a bag similar in size and shape to one later found among Noah's belongings.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Anyone sitting down at that terminal would have had full access without ever needing his password.</t>
+          <t>Combined with the exit-then-reentry pattern, this places someone matching Noah back inside minutes before the badge was used.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>True, but misleading</t>
+          <t>Supporting, not conclusive alone</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>F2, A2</t>
+          <t>E2, B1</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>Noah</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>The first leaked video matches the internal Helix demo.</t>
+          <t>Olivia's device connected to an external file-sharing service shortly before 11:54 PM.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>File comparison shows no added clips or major modification before the first upload.</t>
+          <t>The connection timing is consistent with the second upload, not the original 11:47 upload.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Even compression artifacts and audio levels match the internal master file in the unedited sections.</t>
+          <t>The outbound connection at 11:54 PM matches the same file-sharing service, down to the session ID range.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Whoever uploaded the first video did not alter it, they only moved it.</t>
+          <t>Olivia's device was actively uploading at the exact minute the second video appeared.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1409,270 +1413,270 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>B1, D1</t>
+          <t>F8, A2</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Noah</t>
+          <t>Olivia</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>The second video uses different encoding settings from the first.</t>
+          <t>The security engineer's own system logs are the most complete record of the night, since she personally maintains the logging infrastructure.</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Metadata suggests the additional segment was edited on a different device shortly before 11:54 PM.</t>
+          <t>As the security engineer, Avery configured and maintains every log referenced in this investigation.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>The encoding profile matches a specific video editing application, not the format used for internal demo recordings.</t>
+          <t>That gives her more technical opportunity than anyone else in the building.</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>That application is installed on exactly one company device.</t>
+          <t>But the (independently cross-checked) logs show no tampering or gaps around her own account.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True, but shows opportunity, not guilt</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>G4, C2</t>
+          <t>F1, C2</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Olivia</t>
+          <t>Avery</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F7</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>The security engineer had administrator access to almost every system involved.</t>
+          <t>An unrelated security incident from six months ago turned up in the same server logs.</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>No logs show Avery using privileged access during the relevant period.</t>
+          <t>The log viewer surfaces an entry from an old badge-cloning incident, unconnected to Project Helix.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Her admin credentials were not used to touch any Helix-related file, folder, or system that night.</t>
+          <t>That earlier incident was already resolved, and the employee involved no longer works at the company.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Having the keys to every door is not evidence of walking through one.</t>
+          <t>It only appears in this report because the logging system wasn't filtered by date.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>True, but low relevance</t>
+          <t>Unrelated, resolved</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Low / Red Herring</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>H4, A3</t>
-        </is>
-      </c>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Avery</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>An unrelated security incident from six months ago turned up in the same server logs.</t>
+          <t>Ethan's account accessed the confidential Project Helix folder at 11:39 PM.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>The log viewer surfaces an entry from an old badge-cloning incident, unconnected to Project Helix.</t>
+          <t>No new password was entered. The workstation had already been logged into Ethan's account.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>That earlier incident was already resolved, and the employee involved no longer works at the company.</t>
+          <t>The session had begun over an hour earlier, before Ethan left for his call.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>It only appears in this report because the logging system wasn't filtered by date.</t>
+          <t>Anyone sitting down at that terminal would have had full access without ever needing his password.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Unrelated, resolved</t>
+          <t>True, but misleading</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>E1, E8</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ethan</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>H3</t>
+          <t>H7</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>The lead researcher opposed the Project Helix launch and wanted it delayed.</t>
+          <t>The first leaked video matches the internal Helix demo.</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Internal messages show Ethan repeatedly raised safety concerns about releasing the model too early.</t>
+          <t>File comparison shows no added clips or major modification before the first upload.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>He proposed delaying the launch by at least two weeks, in a message sent to the whole leadership team.</t>
+          <t>Even compression artifacts and audio levels match the internal master file in the unedited sections.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Leadership rejected the delay in writing, giving Ethan a documented but overruled grievance.</t>
+          <t>Whoever uploaded the first video did not alter it, they only moved it.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>True, but motive alone proves nothing</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Medium / Red Herring</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>B2, C1, A1</t>
+          <t>H1, F8</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>Noah</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>A8</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Noah was near Ethan's belongings before the unauthorized Lab 3 entry.</t>
+          <t>The product lead strongly wanted the launch to continue.</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Noah had an opportunity to take Ethan's badge before 11:31 PM.</t>
+          <t>Internal messages show she feared a delay would jeopardize a major launch and partnership.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Noah was seen near the jacket rack by the lab entrance at 11:22 PM, six minutes after Ethan left it there.</t>
+          <t>She wrote that a delay 'could cost us the partnership entirely,' three days before the leak.</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>No one else is placed near that rack in the eleven minutes before the badge was used.</t>
+          <t>Discrediting the leak, not stopping it, would have been enough to save the launch.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>True / Motive</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>E1, G1, B1</t>
+          <t>A2, D7</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Noah</t>
+          <t>Olivia</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>B8</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Olivia's device connected to an external file-sharing service shortly before 11:54 PM.</t>
+          <t>The security engineer was the one who discovered the leak had occurred and escalated it immediately.</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>The connection timing is consistent with the second upload, not the original 11:47 upload.</t>
+          <t>Server monitoring alerts show Avery's account was first to flag anomalous outbound traffic at 11:49 PM.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>The outbound connection at 11:54 PM matches the same file-sharing service, down to the session ID range.</t>
+          <t>She escalated to her manager within two minutes of the alert, well before the video went viral.</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Olivia's device was actively uploading at the exact minute the second video appeared.</t>
+          <t>Someone trying to cover their tracks is not usually the one who raises the alarm.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1682,96 +1686,96 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>D1, C2</t>
+          <t>E1, C2</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Olivia</t>
+          <t>Avery</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C8</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>The security engineer flagged unusual login patterns days before the leak, but was told the issue was low priority.</t>
+          <t>The two leaked videos probably came from the same person because they appeared seven minutes apart.</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>An internal ticket shows Avery reported suspicious badge-sharing behavior three days before the incident.</t>
+          <t>File structure, editing metadata, and upload behavior indicate two separate actions.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Management marked the ticket 'low priority, revisit next quarter.'</t>
+          <t>The two uploads used different devices and different accounts.</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>The exact vulnerability she flagged, a badge used without its owner present, is what let the leak happen.</t>
+          <t>Two people made two separate decisions, seven minutes apart, for two different reasons.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>False assumption</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>H4</t>
+          <t>H7, F8, D1</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Avery</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>The two leaked videos probably came from the same person because they appeared seven minutes apart.</t>
+          <t>Ethan's badge, account, and network location all independently point to Ethan.</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>File structure, editing metadata, and upload behavior indicate two separate actions.</t>
+          <t>All three signals could result from one person using Ethan's badge and already-authenticated workstation inside Lab 3.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>The two uploads used different devices and different accounts.</t>
+          <t>Security consultants confirm this exact scenario, badge theft plus an unlocked terminal, has happened before elsewhere.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Two people made two separate decisions, seven minutes apart, for two different reasons.</t>
+          <t>Three suspicious signals near the same name is not the same thing as three independent proofs.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>False assumption</t>
+          <t>False combined inference</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -1781,44 +1785,44 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>D3, D1, E3</t>
+          <t>C1, G7, E1</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ethan</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>E8</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Ethan's badge, account, and network location all independently point to Ethan.</t>
+          <t>The Lab 3 workstation remained logged into Ethan's account after Ethan left.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>All three signals could result from one person using Ethan's badge and already-authenticated workstation inside Lab 3.</t>
+          <t>Someone could access Project Helix without knowing Ethan's password.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Security consultants confirm this exact scenario, badge theft plus an unlocked terminal, has happened before elsewhere.</t>
+          <t>The workstation's session timeout is set to 60 minutes, unusually long for a machine handling confidential files.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Three suspicious signals near the same name is not the same thing as three independent proofs.</t>
+          <t>That single configuration gap is what turned a forgotten badge into a full breach.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>False combined inference</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1828,194 +1832,147 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>E1, C3, F2</t>
+          <t>G7, B1</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>Noah</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F8</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>The contractor's badge indicates that he had already left the building.</t>
+          <t>A second version of the leaked video appeared online at 11:54 PM.</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>His own badge was used to exit, but a loading-dock camera suggests he later re-entered behind another employee.</t>
+          <t>The second file contains an additional segment not present in the original upload.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>The exit swipe was logged at 9:58 PM, over an hour before the leak.</t>
+          <t>The added segment runs 47 seconds and shows a fabricated 'unsafe response' clip.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>An exit swipe only proves he left once, it says nothing about whether he came back.</t>
+          <t>Someone had access to the original leaked file and editing tools within those seven minutes.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>True record, misleading conclusion</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>A4, G2</t>
+          <t>H7, G2</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Noah</t>
+          <t>Olivia</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>G8</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>The additional unsafe-response clip appears to be part of Project Helix.</t>
+          <t>Avery's badge and login activity that night were both located at her desk on a different floor.</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>The clip does not exist anywhere in the original internal demo.</t>
+          <t>Badge logs show Avery working from her own desk on the third floor from 10 PM until after midnight.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Engineers who ran the original demo confirm the model never produced that response in any recorded session.</t>
+          <t>Her login sessions during that window match routine end-of-day security patch work, unrelated to Lab 3 or Helix.</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>The clip was created separately and spliced in, it did not come from Project Helix at all.</t>
+          <t>None of her recorded activity overlaps with the Lab 3 access window at all.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>False / Manipulated</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>D1, E3</t>
+          <t>F1, C2</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Olivia</t>
+          <t>Avery</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>H4</t>
+          <t>H8</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>The security engineer previously warned that the building's identity and access systems were insecure.</t>
+          <t>A one-day visitor badge was issued earlier that day to an outside vendor unrelated to the four people still in the building.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Her warnings specifically mention badge sharing and unattended authenticated workstations.</t>
+          <t>Front desk logs show the visitor badge was issued at 2 PM for a scheduled equipment demo.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>She filed that warning eleven days before the leak, describing this exact scenario almost precisely.</t>
+          <t>The visitor signed out at 5:30 PM, well before the incident window began.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>The vulnerability she predicted is the one that was actually used, just not by her.</t>
+          <t>Their badge was deactivated at sign-out and was never used again that night.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>True and relevant context</t>
+          <t>TRUE, but irrelevant</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>E1, A2</t>
-        </is>
-      </c>
+          <t>Low / Red Herring</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>Avery</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>A5</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Someone ordered late-night food delivery to the building's side entrance at 11:15 PM.</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>A delivery service confirms a drop-off at the side entrance twenty minutes before the badge swipe.</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Building logs show the side entrance door was propped open for about six minutes around that delivery.</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>No badge or camera record identifies who received the delivery.</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Unverified, no clear connection</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2032,7 +1989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2048,7 +2005,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>(preview: which suspect lands on each square, row-major)</t>
+          <t>(preview: pieces sit on ranks 1-2 and 7-8 only, 3-6 empty)</t>
         </is>
       </c>
     </row>
@@ -2090,14 +2047,14 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>— (H1)</t>
+          <t>Noah (H1)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Noah (A2)</t>
+          <t>Olivia (A2)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2107,17 +2064,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Olivia (C2)</t>
+          <t>Avery (C2)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Avery (D2)</t>
+          <t>— (D2)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>— (E2)</t>
+          <t>Noah (E2)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -2127,105 +2084,37 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Noah (G2)</t>
+          <t>Olivia (G2)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Olivia (H2)</t>
+          <t>Avery (H2)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Avery (A3)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>— (B3)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Ethan (C3)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Noah (D3)</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Olivia (E3)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Avery (F3)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>— (G3)</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Ethan (H3)</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Noah (A4)</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Olivia (B4)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Avery (C4)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>— (D4)</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Ethan (E4)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Noah (F4)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Olivia (G4)</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Avery (H4)</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>— (A5)</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
@@ -2233,6 +2122,100 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>— (A7)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ethan (B7)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Noah (C7)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Olivia (D7)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Avery (E7)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>— (F7)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Ethan (G7)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Noah (H7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Olivia (A8)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Avery (B8)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>— (C8)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ethan (D8)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Noah (E8)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Olivia (F8)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Avery (G8)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>— (H8)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2245,7 +2228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2281,7 +2264,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B2, C1, G1</t>
+          <t>B7, F2, G1</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2279,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A4, A2, B1, D3, G2</t>
+          <t>B1, E8, H1, H7, C7</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2294,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>D1, E3, C2, B4, H2</t>
+          <t>F8, D1, A2, D7, A8</t>
         </is>
       </c>
     </row>
@@ -2326,19 +2309,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>H4, A3, C4, F1, D2</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Dropped: E03 (redundant with E02's badge point), E05 (redundant with E04), E26/E27 (redundant extra alibi pieces).</t>
+          <t>C2, G8, H2, B8, E7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cut Ethan's share and stop two cards giving their suspect away
- "Ethan's Objection" is now "Launch Objection" and reads "Someone on the
  team opposed the launch"; "Noah's Opportunity" is now "Near the Coat
  Rack" and reads "Someone was seen by the jackets and bags...". Digging in
  is what names Ethan / Noah.
- Ethan drops from 9 evidence items to 7 (Noah, Olivia and Avery have 6):
  removed the redundant video-call-witnesses item and re-tagged Upload
  Origin, which names nobody, as neutral. A new low-relevance red herring
  (parking gate glitch) takes the freed square, so the deck stays at 32
  with 7 neutral items.
- data/leakdata.xlsx kept in sync (rows, connects-to, suspect column,
  summary and board-layout sheets).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/leakdata.xlsx
+++ b/data/leakdata.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>The lead researcher opposed the Project Helix launch and wanted it delayed.</t>
+          <t>Someone on the team opposed the Project Helix launch and wanted it delayed.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>B7, F2, B2</t>
+          <t>B7, B2</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -545,12 +545,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Noah was near Ethan's belongings before the unauthorized Lab 3 entry.</t>
+          <t>Someone was seen by the jackets and bags near the Lab 3 entrance shortly before the unauthorized entry.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Noah had an opportunity to take Ethan's badge before 11:31 PM.</t>
+          <t>It was Noah, and he had an opportunity to take Ethan's badge before 11:31 PM.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1105,42 +1105,38 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Ethan was visibly present on the video call.</t>
+          <t>The parking garage gate logged an unusually long open cycle around 11:10 PM.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Multiple participants confirm seeing and speaking with him during the period when Lab 3 was accessed.</t>
+          <t>Facility logs show the barrier stayed raised for four minutes.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Two separate colleagues recall Ethan answering a direct question at 11:38 PM, one minute before the folder was accessed.</t>
+          <t>The gate's sensor had already been reported faulty twice that month.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>It is not physically possible to be speaking on camera and typing in Lab 3 at the same instant.</t>
+          <t>Its timing lines up with nothing else in the investigation.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Coincidence</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>B7, C1, G7</t>
-        </is>
-      </c>
+          <t>Low / Red Herring</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1315,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>C1, F2</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -2032,7 +2028,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Ethan (E1)</t>
+          <t>— (E1)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2079,7 +2075,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Ethan (F2)</t>
+          <t>— (F2)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2093,46 +2089,10 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-    </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -2260,11 +2220,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B7, F2, G1</t>
+          <t>B7, G1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rewrite The Leak evidence so first layers are vague and detail deepens per dig
Base text and labels no longer name suspects or state conclusions; names, times
and exact locations appear only in deeper layers (1-3 per item). Each suspect now
has 7 related items with 4 general ones. Adds the hallway camera and the
contractor's contract status, fixes timeline conflicts, and mirrors the changes
in data/leakdata.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/leakdata.xlsx
+++ b/data/leakdata.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Board Layout" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Board Layout" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -498,22 +498,22 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>The lead researcher opposed the Project Helix launch and wanted it delayed.</t>
+          <t>A senior researcher had voiced strong reservations about the launch timeline.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Internal messages show Ethan repeatedly raised safety concerns about releasing the model too early.</t>
+          <t>Internal messages show the concerns were about safety results not being ready for public release.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>He proposed delaying the launch by at least two weeks, in a message sent to the whole leadership team.</t>
+          <t>Ethan Cole proposed delaying the launch by at least two weeks, in a message sent to the whole leadership team.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Leadership rejected the delay in writing, giving Ethan a documented but overruled grievance.</t>
+          <t>Leadership declined the delay in writing, so his objection is on record as overruled.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -545,22 +545,22 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Noah was near Ethan's belongings before the unauthorized Lab 3 entry.</t>
+          <t>Someone was seen near the coat rack outside a restricted lab shortly before an unexpected entry.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Noah had an opportunity to take Ethan's badge before 11:31 PM.</t>
+          <t>A colleague passing the lab entrance noticed a person lingering by the coat rack.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Noah was seen near the jacket rack by the lab entrance at 11:22 PM, six minutes after Ethan left it there.</t>
+          <t>Noah Reed was seen near the jacket rack at 11:26 PM, about six minutes after Ethan Cole walked out of the lab.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>No one else is placed near that rack in the eleven minutes before the badge was used.</t>
+          <t>No one else is recorded near that rack between 11:20 PM and the badge entry at 11:31 PM.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -592,22 +592,22 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Ethan's badge entered Lab 3 at 11:31 PM.</t>
+          <t>The building's access system logged an entry into a restricted lab late that night.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>The access system records the credential used, not the identity of the person carrying it.</t>
+          <t>The entry was logged against a staff badge credential at one of the lab's door readers.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Facilities confirms badge readers have no camera or biometric check attached to them.</t>
+          <t>The record reads: Ethan Cole — Lab 3 — 11:31 PM. Facilities confirms the readers have no camera or biometric check.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>The log entry only proves the badge was there, not that Ethan was.</t>
+          <t>The swipe was logged as a normal authorized entry, with no failed attempt beforehand and no alarm.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>B7, G1</t>
+          <t>B7, G7, F7</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -639,17 +639,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>The second video uses different encoding settings from the first.</t>
+          <t>The two leaked videos were analyzed for differences in how they were encoded.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Metadata suggests the additional segment was edited on a different device shortly before 11:54 PM.</t>
+          <t>The second video's added segment uses different encoding settings from the rest of the file.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>The encoding profile matches a specific video editing application, not the format used for internal demo recordings.</t>
+          <t>The profile matches a commercial video-editing application, not the format used for internal demo recordings.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -686,22 +686,22 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>The original leaked video was uploaded at 11:47 PM from Lab 3's network.</t>
+          <t>The first leaked video was uploaded from a network inside the building.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Network records identify the location of the connection, not the individual using it.</t>
+          <t>Network records place the upload at 11:47 PM on Lab 3's network.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Lab 3's Wi-Fi range extends into the adjacent break room and stairwell, neither of which needs a badge.</t>
+          <t>Those records identify the location of the connection, not the person using it.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>The upload could have originated from anyone in that wider radius, not only someone inside the locked lab.</t>
+          <t>Lab 3's Wi-Fi range extends into the adjacent break room and stairwell, neither of which requires a badge.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -733,24 +733,20 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>The security engineer had administrator access to almost every system involved.</t>
+          <t>Someone in the building holds administrator rights across most internal systems.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>No logs show Avery using privileged access during the relevant period.</t>
+          <t>A member of the security team has admin credentials for nearly every system involved.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Her admin credentials were not used to touch any Helix-related file, folder, or system that night.</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Having the keys to every door is not evidence of walking through one.</t>
-        </is>
-      </c>
+          <t>Avery Chen's admin credentials were not used on any Helix-related file, folder or system that night.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>True, but low relevance</t>
@@ -780,22 +776,22 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Ethan later reported that his badge had been missing.</t>
+          <t>A staff member later reported a missing access badge.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Ethan last remembers having it before leaving Lab 3 earlier that evening.</t>
+          <t>The report says the badge was last seen in a jacket left near a lab entrance earlier that evening.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>He reported it missing to Avery's team at 11:56 PM, nine minutes after the leak.</t>
+          <t>Ethan Cole filed it with the security team at 11:56 PM, three minutes after his video call ended.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>He reported it before he had any way of knowing a leak had even happened.</t>
+          <t>The report came before security had asked anyone to account for their badge.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -827,22 +823,22 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>A temporary storage device found among a contractor's belongings contains traces of the Helix file structure.</t>
+          <t>A small storage device turned up during a search of personal belongings.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>File timestamps are consistent with the period immediately before the 11:47 PM upload.</t>
+          <t>It holds traces of the same file structure as the Helix demo folder.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>The device shows the Helix demo file copied at 11:41 PM, then deleted from the device at 11:48 PM.</t>
+          <t>File timestamps show the demo file was copied to it at 11:41 PM and removed at 11:48 PM.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Records tie the device to Noah, and the copy-then-delete pattern matches someone erasing their tracks right after uploading.</t>
+          <t>Serial records tie the device to equipment issued to Noah Reed.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -874,22 +870,22 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Olivia's laptop contains the editing environment consistent with the altered video.</t>
+          <t>A company laptop shows activity from a video-editing application around the time of the second upload.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Software activity shows editing shortly before the second upload.</t>
+          <t>The application's autosave history shows a project file opened at 11:49 PM.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>The application's autosave history shows a project file opened at 11:44 PM and exported at 11:53 PM.</t>
+          <t>The same project was exported at 11:53 PM, one minute before the second video appeared online.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>That is the exact editing application and window identified in the encoding metadata.</t>
+          <t>The laptop is Olivia Grant's company-issued device, and the application window matches the one named in the video's encoding metadata.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -921,24 +917,20 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>An anonymous tip claimed Ethan bragged about the leak in a private chat.</t>
+          <t>An anonymous message circulating online claims to reveal who is behind the leak.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>A screenshot circulated online showing a chat message attributed to Ethan admitting to the leak.</t>
+          <t>It includes a screenshot of a chat message attributed to Ethan, in which he appears to admit to the leak.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Metadata on the screenshot shows it was created and edited after the leak had already gone viral.</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>The account named in the screenshot does not match any of Ethan's real usernames, the message was fabricated.</t>
-        </is>
-      </c>
+          <t>The screenshot's metadata shows it was created and edited after the leak was already spreading, and the username in it matches none of Ethan's registered accounts.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>False / Fabricated</t>
@@ -951,7 +943,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>D8, A1</t>
+          <t>A1, C1</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -968,22 +960,22 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>The security engineer previously warned that the building's identity and access systems were insecure.</t>
+          <t>A written warning about the building's identity and access systems was filed before the incident.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Her warnings specifically mention badge sharing and unattended authenticated workstations.</t>
+          <t>It was filed eleven days before the leak and describes the systems as insecure.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>She filed that warning eleven days before the leak, describing this exact scenario almost precisely.</t>
+          <t>Avery Chen's warning specifically mentions badge sharing and unattended authenticated workstations.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>The vulnerability she predicted is the one that was actually used, just not by her.</t>
+          <t>The scenario it describes matches how a badge and a logged-in workstation were used in Lab 3 that night.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1015,24 +1007,16 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>The building's thermostat logged an unusual temperature drop in Lab 3 around midnight.</t>
+          <t>The building's environmental system logged a change in one of the labs around midnight.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Facilities data shows the room cooled by four degrees starting at 11:40 PM.</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Maintenance says this matches a routine HVAC cycle that runs every night at that time.</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>The timing is coincidental and unrelated to anyone's presence.</t>
-        </is>
-      </c>
+          <t>Facilities data shows Lab 3 cooled by four degrees starting at 11:40 PM, and maintenance lists a scheduled nightly cycle for that zone at the same time.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Coincidence</t>
@@ -1043,7 +1027,11 @@
           <t>Low / Red Herring</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -1058,22 +1046,22 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>The contractor's badge indicates that he had already left the building.</t>
+          <t>A badge record shows someone leaving the building earlier that evening.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>His own badge was used to exit, but a loading-dock camera suggests he later re-entered behind another employee.</t>
+          <t>The exit was logged on a contractor badge, and the system shows no later entry on that badge.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>The exit swipe was logged at 9:58 PM, over an hour before the leak.</t>
+          <t>It was Noah Reed's badge, logged at 9:58 PM, nearly two hours before the leak.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>An exit swipe only proves he left once, it says nothing about whether he came back.</t>
+          <t>The loading-dock door has no individual badge reader, so a return through it would leave no badge record.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1105,22 +1093,22 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Ethan was visibly present on the video call.</t>
+          <t>Several colleagues joined a late-night video call with an outside research group.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Multiple participants confirm seeing and speaking with him during the period when Lab 3 was accessed.</t>
+          <t>Participants say one of the researchers was visibly on camera for most of the meeting.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Two separate colleagues recall Ethan answering a direct question at 11:38 PM, one minute before the folder was accessed.</t>
+          <t>Two colleagues recall Ethan Cole answering a direct question at 11:38 PM.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>It is not physically possible to be speaking on camera and typing in Lab 3 at the same instant.</t>
+          <t>One adds that the exchange ran into the next minute, the same minute the Helix folder was accessed from Lab 3.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1152,22 +1140,22 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>The additional unsafe-response clip appears to be part of Project Helix.</t>
+          <t>The second video contains a short clip showing the model giving an unsafe response.</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>The clip does not exist anywhere in the original internal demo.</t>
+          <t>The clip does not appear anywhere in the original internal demo recording.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Engineers who ran the original demo confirm the model never produced that response in any recorded session.</t>
+          <t>Engineers who ran the original demo say the model never produced that response in any recorded session.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>The clip was created separately and spliced in, it did not come from Project Helix at all.</t>
+          <t>Frame and audio analysis show the clip was inserted into the file after the rest of the video had been assembled.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1199,24 +1187,20 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>The security engineer flagged unusual login patterns days before the leak, but was told the issue was low priority.</t>
+          <t>A support ticket about unusual login behavior was opened a few days before the incident.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>An internal ticket shows Avery reported suspicious badge-sharing behavior three days before the incident.</t>
+          <t>The ticket, opened three days before the leak, reports suspicious badge-sharing behavior.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Management marked the ticket 'low priority, revisit next quarter.'</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>The exact vulnerability she flagged, a badge used without its owner present, is what let the leak happen.</t>
-        </is>
-      </c>
+          <t>Avery Chen filed it, and management marked it 'low priority, revisit next quarter.'</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -1246,38 +1230,42 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>A rumor circulated that someone had been secretly recording internal meetings for weeks.</t>
+          <t>One of the people in the building that night had recently received difficult news about their employment.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Two employees mention hearing this rumor in the days before the leak.</t>
+          <t>A temporary contractor was told his contract would not be renewed after the launch.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Neither can say where the rumor started.</t>
+          <t>Noah Reed had also been turned down for a permanent position a few weeks earlier.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Security finds no evidence any meeting was ever recorded without consent.</t>
+          <t>In a message to a colleague, he complained that his work on Helix would be presented without crediting him.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Unsubstantiated rumor</t>
+          <t>True, but motive alone proves nothing</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Low / Red Herring</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>B1, H1</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Noah</t>
         </is>
       </c>
     </row>
@@ -1289,22 +1277,22 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Ethan says he was on a video call during the incident.</t>
+          <t>The company's meeting platform holds a record of a video call that ran through the time of the incident.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Meeting records show Ethan joined at 11:24 PM and remained connected until about 11:53 PM.</t>
+          <t>The platform shows one participant joined from a conference room on a different floor.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>The call platform logs an unbroken connection, no drops and no rejoins, for the full 29 minutes.</t>
+          <t>Ethan Cole joined at 11:24 PM and stayed connected until about 11:53 PM.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>That window fully covers the badge swipe, the folder access, and the upload.</t>
+          <t>The connection log shows no drops and no rejoins across those 29 minutes.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1336,22 +1324,22 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Loading-dock footage shows someone resembling Noah returning to the building.</t>
+          <t>Camera footage from the loading area shows a figure entering the building.</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Clothing and build are consistent with Noah, but the face is only partially visible.</t>
+          <t>The figure came in at 11:09 PM behind another employee who held open a door that needs no individual badge.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
+          <t>Clothing and build are consistent with Noah Reed, but the face is only partly visible.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
           <t>The figure carries a bag similar in size and shape to one later found among Noah's belongings.</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Combined with the exit-then-reentry pattern, this places someone matching Noah back inside minutes before the badge was used.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1383,22 +1371,22 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Olivia's device connected to an external file-sharing service shortly before 11:54 PM.</t>
+          <t>Network records show a company device connecting to an outside file-sharing service late that night.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>The connection timing is consistent with the second upload, not the original 11:47 upload.</t>
+          <t>The connection opened shortly before 11:54 PM, not in the window around the first upload at 11:47 PM.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>The outbound connection at 11:54 PM matches the same file-sharing service, down to the session ID range.</t>
+          <t>The session matches the file-sharing service the second video was posted through, down to the session ID range.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Olivia's device was actively uploading at the exact minute the second video appeared.</t>
+          <t>The device is registered to Olivia Grant and was still uploading at 11:54 PM.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1430,24 +1418,20 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>The security engineer's own system logs are the most complete record of the night, since she personally maintains the logging infrastructure.</t>
+          <t>Most of the night's records come from a single logging system.</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>As the security engineer, Avery configured and maintains every log referenced in this investigation.</t>
+          <t>The security engineer configured and maintains the logging infrastructure behind every log used in this review.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>That gives her more technical opportunity than anyone else in the building.</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>But the (independently cross-checked) logs show no tampering or gaps around her own account.</t>
-        </is>
-      </c>
+          <t>An independent cross-check of the logs found no tampering and no gaps around her own account.</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
           <t>True, but shows opportunity, not guilt</t>
@@ -1477,35 +1461,39 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>An unrelated security incident from six months ago turned up in the same server logs.</t>
+          <t>Security footage shows a person entering a hallway near the lab.</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>The log viewer surfaces an entry from an old badge-cloning incident, unconnected to Project Helix.</t>
+          <t>The clip is timestamped 11:33 PM, two minutes after the lab entry record.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>That earlier incident was already resolved, and the employee involved no longer works at the company.</t>
+          <t>The person wears a dark company hoodie, the same style Ethan Cole and several other staff own.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>It only appears in this report because the logging system wasn't filtered by date.</t>
+          <t>The camera never captures a clear view of the face.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Unrelated, resolved</t>
+          <t>True, but misleading</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr"/>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>C1, G7</t>
+        </is>
+      </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -1520,22 +1508,22 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Ethan's account accessed the confidential Project Helix folder at 11:39 PM.</t>
+          <t>The confidential demo folder was opened from a lab workstation during the evening.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>No new password was entered. The workstation had already been logged into Ethan's account.</t>
+          <t>The log attributes the access to a user account, with no fresh login event.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>The session had begun over an hour earlier, before Ethan left for his call.</t>
+          <t>Ethan Cole's account accessed the Helix folder at 11:39 PM, and no password was entered at that time.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Anyone sitting down at that terminal would have had full access without ever needing his password.</t>
+          <t>The workstation's session had already been active for more than an hour before the access.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1567,22 +1555,22 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>The first leaked video matches the internal Helix demo.</t>
+          <t>The first leaked video was compared against the company's internal demo recording.</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>File comparison shows no added clips or major modification before the first upload.</t>
+          <t>The comparison finds no added or removed clips.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Even compression artifacts and audio levels match the internal master file in the unedited sections.</t>
+          <t>Compression artifacts and audio levels match the internal master file in every section.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Whoever uploaded the first video did not alter it, they only moved it.</t>
+          <t>The file's metadata shows it was copied from the internal demo shortly before the 11:47 PM upload.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1614,22 +1602,22 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>The product lead strongly wanted the launch to continue.</t>
+          <t>One team member pushed hard to keep the launch on schedule.</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Internal messages show she feared a delay would jeopardize a major launch and partnership.</t>
+          <t>Internal messages show concern that a delay would put a major partnership at risk.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>She wrote that a delay 'could cost us the partnership entirely,' three days before the leak.</t>
+          <t>Olivia Grant wrote that a delay 'could cost us the partnership entirely,' three days before the leak.</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Discrediting the leak, not stopping it, would have been enough to save the launch.</t>
+          <t>In the same thread she argued that the open safety findings could be addressed after release.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1661,22 +1649,22 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>The security engineer was the one who discovered the leak had occurred and escalated it immediately.</t>
+          <t>An automated alert about unusual outbound traffic was raised that night.</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Server monitoring alerts show Avery's account was first to flag anomalous outbound traffic at 11:49 PM.</t>
+          <t>The alert fired at 11:49 PM and was picked up first by the security team's monitoring account.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>She escalated to her manager within two minutes of the alert, well before the video went viral.</t>
+          <t>Avery Chen escalated it to her manager within two minutes of the alert.</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Someone trying to cover their tracks is not usually the one who raises the alarm.</t>
+          <t>That was before the video began spreading widely online.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1708,32 +1696,32 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>The two leaked videos probably came from the same person because they appeared seven minutes apart.</t>
+          <t>Both leaked videos were posted anonymously through public file-sharing services.</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>File structure, editing metadata, and upload behavior indicate two separate actions.</t>
+          <t>The two uploads came from different accounts, each created within the hour before posting.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>The two uploads used different devices and different accounts.</t>
+          <t>They were sent from different networks: the first from Lab 3's network, the second from a device elsewhere in the building.</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Two people made two separate decisions, seven minutes apart, for two different reasons.</t>
+          <t>No login, device or network detail is shared between the two uploads.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>False assumption</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1743,7 +1731,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Olivia</t>
         </is>
       </c>
     </row>
@@ -1755,42 +1743,38 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Ethan's badge, account, and network location all independently point to Ethan.</t>
+          <t>An older security incident report appeared in the same system logs pulled for this review.</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>All three signals could result from one person using Ethan's badge and already-authenticated workstation inside Lab 3.</t>
+          <t>It describes a badge-cloning incident from six months earlier.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Security consultants confirm this exact scenario, badge theft plus an unlocked terminal, has happened before elsewhere.</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>Three suspicious signals near the same name is not the same thing as three independent proofs.</t>
-        </is>
-      </c>
+          <t>The security team handled it and closed it at the time, and the employee involved has since left the company.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>False combined inference</t>
+          <t>Unrelated, resolved</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>C1, G7, E1</t>
+          <t>None</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>Avery</t>
         </is>
       </c>
     </row>
@@ -1802,22 +1786,22 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>The Lab 3 workstation remained logged into Ethan's account after Ethan left.</t>
+          <t>A shared lab workstation was left in an active session that evening.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Someone could access Project Helix without knowing Ethan's password.</t>
+          <t>The machine's session timeout is set to 60 minutes, longer than most machines that handle confidential files.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>The workstation's session timeout is set to 60 minutes, unusually long for a machine handling confidential files.</t>
+          <t>The session was opened under Ethan Cole's account before he left for his call.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>That single configuration gap is what turned a forgotten badge into a full breach.</t>
+          <t>With the session already authenticated, anyone sitting down there could open Helix files without a password.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1849,22 +1833,22 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>A second version of the leaked video appeared online at 11:54 PM.</t>
+          <t>A second version of the leaked video appeared online a few minutes after the first.</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>The second file contains an additional segment not present in the original upload.</t>
+          <t>The second file contains an additional segment that is not in the original upload.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>The added segment runs 47 seconds and shows a fabricated 'unsafe response' clip.</t>
+          <t>The added segment runs 47 seconds and shows an unsafe model response.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Someone had access to the original leaked file and editing tools within those seven minutes.</t>
+          <t>Adding it required a copy of the leaked file and editing tools within the seven minutes after the first upload.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1896,22 +1880,22 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Avery's badge and login activity that night were both located at her desk on a different floor.</t>
+          <t>Badge and login records place a staff member on a different floor throughout the incident window.</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Badge logs show Avery working from her own desk on the third floor from 10 PM until after midnight.</t>
+          <t>Badge logs show a security engineer at her own desk on the third floor from 10 PM until after midnight.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Her login sessions during that window match routine end-of-day security patch work, unrelated to Lab 3 or Helix.</t>
+          <t>Avery Chen's login sessions in that period match routine end-of-day security patch work.</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>None of her recorded activity overlaps with the Lab 3 access window at all.</t>
+          <t>None of her recorded activity overlaps with the Lab 3 entry at 11:31 PM or the folder access at 11:39 PM.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1943,24 +1927,20 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>A one-day visitor badge was issued earlier that day to an outside vendor unrelated to the four people still in the building.</t>
+          <t>A one-day visitor badge was issued earlier that day.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Front desk logs show the visitor badge was issued at 2 PM for a scheduled equipment demo.</t>
+          <t>Front desk logs show it was issued at 2 PM to an outside vendor for a scheduled equipment demo.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>The visitor signed out at 5:30 PM, well before the incident window began.</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Their badge was deactivated at sign-out and was never used again that night.</t>
-        </is>
-      </c>
+          <t>The visitor signed out at 5:30 PM, when the badge was deactivated, and it shows no activity afterward.</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
           <t>TRUE, but irrelevant</t>
@@ -1971,7 +1951,11 @@
           <t>Low / Red Herring</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -2032,7 +2016,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Ethan (E1)</t>
+          <t>— (E1)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2093,50 +2077,14 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-    </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>— (A7)</t>
+          <t>Noah (A7)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2188,12 +2136,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>— (C8)</t>
+          <t>Olivia (C8)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Ethan (D8)</t>
+          <t>Avery (D8)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -2264,7 +2212,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B7, F2, G1</t>
+          <t>G1, F2, B7</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2227,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>B1, E8, H1, H7, C7</t>
+          <t>B1, H1, C7, H7, E8</t>
         </is>
       </c>
     </row>
@@ -2290,11 +2238,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>F8, D1, A2, D7, A8</t>
+          <t>D1, A2, D7, A8, C8, F8</t>
         </is>
       </c>
     </row>
@@ -2309,7 +2257,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>C2, G8, H2, B8, E7</t>
+          <t>C2, H2, E7, B8, G8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Describe desk activity as credential records; mark factual red herrings real
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/leakdata.xlsx
+++ b/data/leakdata.xlsx
@@ -1764,7 +1764,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Low / Red Herring</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1880,12 +1880,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Badge and login records place a staff member on a different floor throughout the incident window.</t>
+          <t>Badge and login records show credential activity on a different floor throughout the incident window.</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Badge logs show a security engineer at her own desk on the third floor from 10 PM until after midnight.</t>
+          <t>Badge logs show a security engineer's badge used at third-floor readers from 10 PM until after midnight.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>None of her recorded activity overlaps with the Lab 3 entry at 11:31 PM or the folder access at 11:39 PM.</t>
+          <t>None of her recorded badge or login activity overlaps with the Lab 3 entry at 11:31 PM or the folder access at 11:39 PM.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2077,10 +2077,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>

</xml_diff>